<commit_message>
fix for github actions
</commit_message>
<xml_diff>
--- a/test-data/excel/testData.xlsx
+++ b/test-data/excel/testData.xlsx
@@ -40,22 +40,22 @@
     <t>EmployeeID</t>
   </si>
   <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Doe</t>
-  </si>
-  <si>
-    <t>0398</t>
+    <t>Jon</t>
+  </si>
+  <si>
+    <t>Bon</t>
+  </si>
+  <si>
+    <t>Jovi</t>
+  </si>
+  <si>
+    <t>0383</t>
   </si>
   <si>
     <t>Status</t>
   </si>
   <si>
-    <t>john.doe29</t>
+    <t>john.doe31</t>
   </si>
   <si>
     <t>P@ssw0rd123</t>

</xml_diff>

<commit_message>
data mutation enable/disable via environment variable
</commit_message>
<xml_diff>
--- a/test-data/excel/testData.xlsx
+++ b/test-data/excel/testData.xlsx
@@ -1,50 +1,116 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="LoginData" sheetId="1" r:id="rId1"/>
-    <sheet name="EmployeeData" sheetId="2" r:id="rId2"/>
-    <sheet name="EmployeeLoginData" sheetId="3" r:id="rId3"/>
-    <sheet name="PersonalDetails" sheetId="4" r:id="rId4"/>
+    <sheet sheetId="1" name="LoginData" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="EmployeeData" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="EmployeeLoginData" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="PersonalDetails" state="visible" r:id="rId7"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>admin123</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>MiddleName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>EmployeeID</t>
+  </si>
+  <si>
+    <t>Jon</t>
+  </si>
+  <si>
+    <t>Bon</t>
+  </si>
+  <si>
+    <t>Jovi</t>
+  </si>
+  <si>
+    <t>0399</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>john.doe32</t>
+  </si>
+  <si>
+    <t>P@ssw0rd123</t>
+  </si>
+  <si>
+    <t>Enabled</t>
+  </si>
+  <si>
+    <t>License</t>
+  </si>
+  <si>
+    <t>LicenseExpiry</t>
+  </si>
+  <si>
+    <t>Nationality</t>
+  </si>
+  <si>
+    <t>MaritalStatus</t>
+  </si>
+  <si>
+    <t>DOB</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>DL-987651</t>
+  </si>
+  <si>
+    <t>2030-12-31</t>
+  </si>
+  <si>
+    <t>Bangladeshi</t>
+  </si>
+  <si>
+    <t>Single</t>
+  </si>
+  <si>
+    <t>1998-06-15</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -68,13 +134,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -399,151 +473,143 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B2"/>
+  <sheetFormatPr customHeight="1"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Username</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Password</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Admin</v>
-      </c>
-      <c r="B2" t="str">
-        <v>admin123</v>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D2"/>
+  <sheetFormatPr customHeight="1"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>FirstName</v>
-      </c>
-      <c r="B1" t="str">
-        <v>MiddleName</v>
-      </c>
-      <c r="C1" t="str">
-        <v>LastName</v>
-      </c>
-      <c r="D1" t="str">
-        <v>EmployeeID</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Jon</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Bon</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Jovi</v>
-      </c>
-      <c r="D2" t="str">
-        <v/>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C2"/>
+  <sheetFormatPr customHeight="1"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Username</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Password</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Status</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>john.doe32</v>
-      </c>
-      <c r="B2" t="str">
-        <v>P@ssw0rd123</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Enabled</v>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F2"/>
+  <sheetFormatPr customHeight="1"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>License</v>
-      </c>
-      <c r="B1" t="str">
-        <v>LicenseExpiry</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Nationality</v>
-      </c>
-      <c r="D1" t="str">
-        <v>MaritalStatus</v>
-      </c>
-      <c r="E1" t="str">
-        <v>DOB</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Gender</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>DL-987651</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2030-12-31</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Bangladeshi</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Single</v>
-      </c>
-      <c r="E2" t="str">
-        <v>1998-06-15</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Male</v>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
OrangeHRM known bug handled
</commit_message>
<xml_diff>
--- a/test-data/excel/testData.xlsx
+++ b/test-data/excel/testData.xlsx
@@ -55,7 +55,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>john.doe32</t>
+    <t>john.doe33</t>
   </si>
   <si>
     <t>P@ssw0rd123</t>
@@ -475,7 +475,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -500,7 +500,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -537,7 +537,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -568,7 +568,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">

</xml_diff>